<commit_message>
Drop the three low-value new connections
Rachael VanLandingham, Anouk Malavoy, and Carly Lund are removed from the new
first-degree batch. The first has a one-word headline with nothing to
personalise against, the second is a Chief AI Officer, and the third sells SaaS.
None supports an honest personalised line for a K-5 picture book.

Their letters are deleted rather than left greyed out, so the sheet contains
only what should actually be sent. Disposition and reason for each are recorded
on the second tab, alongside the eight names already covered in earlier files.

Ten messages remain in this batch. Running total is 626.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bCVQmU5dQHBfkG189ujSG
</commit_message>
<xml_diff>
--- a/CGB_NEW_1st_degree_July.xlsx
+++ b/CGB_NEW_1st_degree_July.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New 1st-degree (Jul 19-27)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Already covered" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="86ed + already covered" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -37,7 +37,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -47,21 +47,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000054A6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,15 +62,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -452,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -461,11 +443,10 @@
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="72" customWidth="1" min="8" max="8"/>
-    <col width="100" customWidth="1" min="9" max="9"/>
+    <col width="74" customWidth="1" min="7" max="7"/>
+    <col width="102" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,25 +482,20 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Send?</t>
+          <t>The skinny</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>The skinny</t>
+          <t>Message (ready to paste)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Message (ready to paste)</t>
+          <t>Sent?</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Sent?</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Reply?</t>
         </is>
@@ -552,23 +528,18 @@
           <t>Jul 25</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>CEO of FCCLA. 257,000+ members, 5,300+ chapters, 49 state associations. Financial literacy is already an active focus (Virtual Business Challenge). The catch: FCCLA is Family &amp; Consumer Sciences, so members are middle and high school, not K-5. The play is not curriculum adoption, it is service projects. FCCLA chapters run community service; a chapter reading Clarence to an elementary class is a ready-made project. Biggest name in this batch by an order of magnitude.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>CEO of FCCLA. 257,000+ members, 5,300+ chapters, 49 state associations. Financial literacy is already an active focus (Virtual Business Challenge). The catch: FCCLA is Family &amp; Consumer Sciences, so members are middle and high school, not K-5. The play is not curriculum adoption, it is service projects. FCCLA chapters run community service; a chapter reading Clarence to an elementary class is a ready-made project. Biggest name in this batch by an order of magnitude.</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
           <t>Sandy — FCCLA members are a decade older than my readers, so this is not a curriculum pitch. It's a service-project one. Your chapters already run community work, and a high schooler reading a money book to a second-grade class is about the cleanest version of that I can think of. Mine is 36 pages, teaches the whole purchase through the register, and the toolkit behind it is free. Does that fit how chapters choose projects, or am I inventing a use case? Toolkit: https://clarencegetsabargain.com/educator-toolkit.html · Sample: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -597,23 +568,18 @@
           <t>Jul 24</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Executive Director, Econiful (Tucson nonprofit, free resources for economics educators). 17 years in the classroom, 2024 NAEE Rising Star, currently building an 80-lesson high school econ curriculum. Econiful serves Grade 6+, so mine sits directly below her band. Complementary rather than competitive, and worth saying so plainly.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Executive Director, Econiful (Tucson nonprofit, free resources for economics educators). 17 years in the classroom, 2024 NAEE Rising Star, currently building an 80-lesson high school econ curriculum. Econiful serves Grade 6+, so mine sits directly below her band. Complementary rather than competitive, and worth saying so plainly.</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
           <t>Megan — Econiful starts at grade 6, which puts my book directly underneath you rather than beside you. Mine is the K-5 on-ramp: a six-year-old runs one purchase, ad to register, sales tax at the end. Congratulations on the Rising Star, by the way. Genuine question rather than a pitch — do you see elementary as in scope for Econiful, or a gap somebody else has to fill? Toolkit: https://clarencegetsabargain.com/educator-toolkit.html · Flip through it: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -642,23 +608,18 @@
           <t>Jul 22</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Founder of CASHVERSE KIDS, 'Building a Story-First Financial Literacy Universe for Kids.' German-speaking (headline reads 'Founder bei'). Not indexed anywhere I can find, so likely pre-launch or very new. Same thesis as yours, stated almost word for word. Closest philosophical peer in the entire list — treat as a peer note, not a pitch.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Founder of CASHVERSE KIDS, 'Building a Story-First Financial Literacy Universe for Kids.' German-speaking (headline reads 'Founder bei'). Not indexed anywhere I can find, so likely pre-launch or very new. Same thesis as yours, stated almost word for word. Closest philosophical peer in the entire list — treat as a peer note, not a pitch.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
           <t>Daniel — 'story-first financial literacy' is my entire thesis too, which is either a good sign or a crowded room. Mine went narrow: one purchase, ad to register, sales tax at the end, 36 pages. Yours sounds like a universe rather than a single trip. Curious whether we are solving the same problem at different scales, or the same scale from different ends. Trade notes? More: https://clarencegetsabargain.com/ · First pages: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -687,23 +648,18 @@
           <t>Jul 23</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Investigative reporter, Chicago Sun-Times. Consumer investigations rather than personal finance columns, so the hook is the category gap, not the book. Pitch the omission and let her decide whether it's a story.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Investigative reporter, Chicago Sun-Times. Consumer investigations rather than personal finance columns, so the hook is the category gap, not the book. Pitch the omission and let her decide whether it's a story.</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
           <t>Stephanie — an investigations angle rather than a book pitch. Children's financial literacy is a real publishing category, and every title in it teaches saving. I read all 25 on the ABA Foundation's list to be sure. None teaches spending, which is the only money thing a six-year-old actually does. Forty years, one blind spot. I wrote the counterexample, but the gap is the more interesting half. Worth a look, or a colleague who'd want it? Press kit: https://clarencegetsabargain.com/press-kit.html · A few pages: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -732,23 +688,18 @@
           <t>Jul 24</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Financial Wellness Lead at Stanford Federal Credit Union. '2026 GAC Crasher' means he was at the Governmental Affairs Conference, so he is plugged into the national credit union scene, not just his own shop. Credit unions are the most likely local funders of K-5 sets.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Financial Wellness Lead at Stanford Federal Credit Union. '2026 GAC Crasher' means he was at the Governmental Affairs Conference, so he is plugged into the national credit union scene, not just his own shop. Credit unions are the most likely local funders of K-5 sets.</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
           <t>Danial — 'making money more human' is a good line, and it happens to be the hardest part of teaching a six-year-old. Mine does it by refusing to be a worksheet: a boy, a robot, one real purchase through the register. There's a grant packet behind it with the math already done, 25 copies at $499.75, in case Stanford FCU ever funds a classroom set. Fit a member or community program? Funding packet: https://clarencegetsabargain.com/resources/grant-in-a-box.html · Preview: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -777,23 +728,18 @@
           <t>Jul 21</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Director of Financial Well-Being, credit union. CCUFC (Certified Credit Union Financial Counselor) and CUDE (Credit Union Development Educator) — the CUDE in particular means she is a movement person, not just a job-holder. Good candidate for the grant-packet angle.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Director of Financial Well-Being, credit union. CCUFC (Certified Credit Union Financial Counselor) and CUDE (Credit Union Development Educator) — the CUDE in particular means she is a movement person, not just a job-holder. Good candidate for the grant-packet angle.</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
           <t>Bree — a CUDE tends to think about the movement rather than the quarter, which is why I'm asking you rather than a marketing desk. Mine is K-5, the band almost nobody builds for, and the whole toolkit is free. There's a grant packet with the math done if a credit union ever wanted to fund a classroom set. Fit your well-being work? Funding packet: https://clarencegetsabargain.com/resources/grant-in-a-box.html · See it: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -822,23 +768,18 @@
           <t>Jul 26</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Director of Product Innovation at Student Connections (student financial services and success). Product lens rather than curriculum lens, so ask her the product question rather than the pedagogy one.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Director of Product Innovation at Student Connections (student financial services and success). Product lens rather than curriculum lens, so ask her the product question rather than the pedagogy one.</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
           <t>Sara — a product innovation question rather than a book pitch. Mine is deliberately low-tech: a printed read-along with free print-ready lessons. No login, no platform, no seats to provision, which either makes it frictionless or makes it a relic. You'd know which. Does analog still work at K-5, or am I fighting the tide? Free toolkit: https://clarencegetsabargain.com/educator-toolkit.html · Sample: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -867,23 +808,18 @@
           <t>Jul 25</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Personal Financial Literacy Coordinator. No employer in the headline, so the message stays on the role rather than the institution. Coordinators are the people who actually have to make a resource work, which is a useful read.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Personal Financial Literacy Coordinator. No employer in the headline, so the message stays on the role rather than the institution. Coordinators are the people who actually have to make a resource work, which is a useful read.</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
           <t>Miche — coordinators are the ones who have to make the thing actually work after somebody else picks it, which is why your read is worth more than a director's. Mine needs no prep, no platform, nothing consumable, and the lessons are free. Four 45-minute plans, a pre/post assessment, a 23-row crosswalk. Would it survive contact with a real schedule? Free toolkit: https://clarencegetsabargain.com/educator-toolkit.html · Flip through it: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -912,23 +848,18 @@
           <t>Jul 24</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>CEO, strategist, podcaster, helicopter pilot, 'Question Asker', 'Creator of Good'. The headline is doing a lot of work and clearly enjoys itself, so match the register. Podcast is the ask.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>CEO, strategist, podcaster, helicopter pilot, 'Question Asker', 'Creator of Good'. The headline is doing a lot of work and clearly enjoys itself, so match the register. Podcast is the ask.</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
           <t>Matt — 'Question Asker' and 'Helicopter Pilot' in the same headline is a choice, and I respect it. Here's a question for you then: every children's money book teaches saving, and not one teaches spending, which is the only money thing a six-year-old actually does. I wrote the one that does. Real gap, or am I picking a fight nobody asked for? Podcast fit, or just curious? More: https://clarencegetsabargain.com/ · First pages: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -957,158 +888,18 @@
           <t>Jul 27</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Financial Literacy Educator and Marketing Professional. The marketing half is the useful half — she can judge positioning, not just content. Newest connection in the batch.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Financial Literacy Educator and Marketing Professional. The marketing half is the useful half — she can judge positioning, not just content. Newest connection in the batch.</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
           <t>Laura — the marketing half of your headline is the half I want. Mine teaches six-year-olds to spend well rather than to save, which puts it in a category of roughly one and makes it awkward to shelve. Educator to marketer: does the positioning work, or does 'the spending book' just confuse people? More: https://clarencegetsabargain.com/ · A few pages: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="n">
-        <v>30</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>7. District / Curriculum</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Rachael VanLandingham</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Educator</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Jul 24</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>MARGINAL</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Headline is one word: 'Educator'. Nothing to personalise against beyond the role itself. Marginal — worth a short honest note rather than a manufactured one, or skip until you know more.</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Rachael — your headline says 'Educator' and nothing else, so I'll skip the fake familiarity. Mine is a K-5 picture book that teaches spending rather than saving, with free zero-prep lessons behind it. If that is nowhere near your grade band, say so and I'll leave you alone. If it's close, I'd value the read. Free toolkit: https://clarencegetsabargain.com/educator-toolkit.html · Preview: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="n">
-        <v>24</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>9. Kids-finance founder</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Anouk Malavoy</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Chief AI Officer (CAIO) | AI Transformation Executive</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Jul 20</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>SKIP unless warming</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Chief AI Officer, AI transformation executive. Off-target for the book, but she is a connection and the book was illustrated with AI tools, which is a genuine and unusual point of contact. Light touch only.</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Anouk — off your beat, but there's one real overlap. I wrote and illustrated a children's book, and the illustration was done with AI tools over about two years of getting a consistent style out of them. The book itself teaches six-year-olds how to spend money well. Either half interest you, or shall I stop there? More: https://clarencegetsabargain.com/ · See it: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="n">
-        <v>20</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>9. Kids-finance founder</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Carly Lund</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Sr. Account Executive | Quota-Carrying SaaS Seller | GTM Leader</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Jul 20</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>SKIP unless warming</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Senior Account Executive, SaaS, GTM. Genuinely off-target — no education, finance-education, or media hook. Lowest value in the batch. Send only if you want the network warm; there is no professional angle here worth manufacturing.</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Carly — nothing to sell you and nothing SaaS about this. I wrote a kids' picture book about spending money well: a boy, a robot, one trip to the register. Thought it might land with a young reader in your world. That's the entire pitch. More: https://clarencegetsabargain.com/ · Sample: https://heyzine.com/flip-book/eeb1ef6cff.html</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1121,103 +912,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>Where</t>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Disposition</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Reason</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Varun Gupta</t>
+          <t>Rachael VanLandingham</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>already written</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>File 2 (199-396)</t>
+          <t>86ed</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Headline is the single word "Educator". Nothing to personalise against.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alyssa Osorio</t>
+          <t>Anouk Malavoy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>already written</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>File 2</t>
+          <t>86ed</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Chief AI Officer. Off-target for a K-5 picture book.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dr. Michael L. James</t>
+          <t>Carly Lund</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>already written</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>File 1 (1-198)</t>
+          <t>86ed</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>SaaS account executive. No education, finance-ed, or media hook.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Kimberly Evans Sulfridge</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>already written</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>File 1</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tobi Amure</t>
+          <t>Varun Gupta</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1225,16 +1004,16 @@
           <t>already written</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>File 2</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>File 2 (199-396)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mart Vainu</t>
+          <t>Alyssa Osorio</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1242,16 +1021,16 @@
           <t>already written</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>File 4 (517-616)</t>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>File 2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wendy Connett</t>
+          <t>Dr. Michael L. James</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1259,24 +1038,92 @@
           <t>already written</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>File 2</t>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>File 1 (1-198)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Kimberly Evans Sulfridge</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>already written</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>File 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tobi Amure</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>already written</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>File 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mart Vainu</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>already written</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>File 4 (517-616)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Wendy Connett</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>already written</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>File 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Kate Dore</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>already written</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>File 1</t>
         </is>
@@ -1293,7 +1140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1301,12 +1148,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>POINT</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DETAIL</t>
         </is>
@@ -1320,7 +1167,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>21 names read off the screenshots. 8 already covered in files 1-4; 13 were new.</t>
+          <t>21 names off the screenshots. 8 already covered in files 1-4, 3 disposed of, 10 written.</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1179,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Sandy Spavone, CEO of FCCLA. 257,000+ members, 5,300+ chapters, 49 state associations, and financial literacy is already an active focus there via the Virtual Business Challenge.</t>
+          <t>Sandy Spavone, CEO of FCCLA. 257,000+ members, 5,300+ chapters, 49 state associations, financial literacy already an active focus via the Virtual Business Challenge.</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1191,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>FCCLA is Family and Consumer Sciences, so members are middle and high school, not K-5. Curriculum would miss. The letter pitches a chapter service project instead: a high schooler reading the book to a second-grade class.</t>
+          <t>FCCLA is Family and Consumer Sciences, so members are middle and high school, not K-5. Curriculum would miss. The letter pitches a chapter service project: a high schooler reading the book to a second-grade class.</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1203,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Daniel Rauen, CASHVERSE KIDS, describes his work as a story-first financial literacy universe for kids. Your thesis, almost word for word. Nothing indexed anywhere, so likely pre-launch. Written as a peer note, not a pitch.</t>
+          <t>Daniel Rauen, CASHVERSE KIDS, a story-first financial literacy universe for kids. Your thesis almost word for word. Nothing indexed anywhere, so likely pre-launch. Written as a peer note.</t>
         </is>
       </c>
     </row>
@@ -1368,43 +1215,31 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Megan Kirts runs Econiful, which serves grade 6 and up, putting your book directly below her band rather than against it. 2024 NAEE Rising Star.</t>
+          <t>Megan Kirts runs Econiful, grade 6 and up, which puts your book below her band rather than against it. 2024 NAEE Rising Star.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Three I would skip</t>
+          <t>Ranking basis</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Rachael VanLandingham (headline is the single word Educator), Anouk Malavoy (Chief AI Officer, though the AI-illustration angle is real), Carly Lund (SaaS sales, no hook). Letters written anyway, flagged red.</t>
+          <t>Reach and gatekeeper power first, then relevance to K-5, then whether the headline supports an honest personalised line.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ranking basis</t>
+          <t>Running total</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Reach and gatekeeper power first, then relevance to K-5, then whether the headline supports an honest personalised line.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Audit</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Same rules as every previous file. No kill-list words, no spoiler leaks, no tired finance puns, no grammar flags, em dashes throughout.</t>
+          <t>626 bespoke messages across five files.</t>
         </is>
       </c>
     </row>

</xml_diff>